<commit_message>
Revert .gitignore change f72cecd2dda901a41f62ea0de572d2292a0545b1
</commit_message>
<xml_diff>
--- a/fix/qa-validation-errors/ig/StructureDefinition-fr-cda-participant-corps.xlsx
+++ b/fix/qa-validation-errors/ig/StructureDefinition-fr-cda-participant-corps.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$36</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="194">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-01T12:39:31+00:00</t>
+    <t>2026-09-03T14:38:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -462,10 +462,25 @@
     <t>Autre TemplateId</t>
   </si>
   <si>
+    <t>Participant2.templateId:templateId-other.nullFlavor</t>
+  </si>
+  <si>
+    <t>Participant2.templateId:templateId-other.assigningAuthorityName</t>
+  </si>
+  <si>
+    <t>Participant2.templateId:templateId-other.displayable</t>
+  </si>
+  <si>
+    <t>Participant2.templateId:templateId-other.root</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Participant2.templateId:templateId-other.extension</t>
+  </si>
+  <si>
     <t>Participant2.typeCode</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
   <si>
     <t>http://hl7.org/cda/stds/core/ValueSet/CDAParticipationType|2.0.3-sd</t>
@@ -915,10 +930,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK31"/>
+  <dimension ref="A1:AK36"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="48.39453125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="53.1484375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="39.30859375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="14.20703125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
@@ -2812,26 +2827,28 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
         <v>145</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E19" s="2"/>
+      <c r="E19" t="s" s="2">
+        <v>85</v>
+      </c>
       <c r="F19" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>146</v>
+        <v>75</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>75</v>
@@ -2843,7 +2860,9 @@
         <v>86</v>
       </c>
       <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
+      <c r="M19" t="s" s="2">
+        <v>87</v>
+      </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -2873,7 +2892,7 @@
       </c>
       <c r="Y19" s="2"/>
       <c r="Z19" t="s" s="2">
-        <v>147</v>
+        <v>89</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>75</v>
@@ -2891,10 +2910,10 @@
         <v>75</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>145</v>
+        <v>90</v>
       </c>
       <c r="AG19" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AH19" t="s" s="2">
         <v>76</v>
@@ -2911,16 +2930,18 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E20" s="2"/>
+      <c r="E20" t="s" s="2">
+        <v>102</v>
+      </c>
       <c r="F20" t="s" s="2">
         <v>81</v>
       </c>
@@ -2937,10 +2958,12 @@
         <v>75</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="M20" t="s" s="2">
+        <v>104</v>
+      </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -2948,7 +2971,7 @@
       </c>
       <c r="Q20" s="2"/>
       <c r="R20" t="s" s="2">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="S20" t="s" s="2">
         <v>75</v>
@@ -2966,11 +2989,13 @@
         <v>75</v>
       </c>
       <c r="X20" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y20" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y20" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z20" t="s" s="2">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>75</v>
@@ -2988,7 +3013,7 @@
         <v>75</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>148</v>
+        <v>105</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -3008,16 +3033,18 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E21" s="2"/>
+      <c r="E21" t="s" s="2">
+        <v>107</v>
+      </c>
       <c r="F21" t="s" s="2">
         <v>81</v>
       </c>
@@ -3034,10 +3061,12 @@
         <v>75</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>152</v>
+        <v>108</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+      <c r="M21" t="s" s="2">
+        <v>109</v>
+      </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -3087,7 +3116,7 @@
         <v>75</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>151</v>
+        <v>110</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
@@ -3107,24 +3136,26 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E22" s="2"/>
+      <c r="E22" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="F22" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>75</v>
@@ -3133,13 +3164,11 @@
         <v>75</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="L22" t="s" s="2">
-        <v>155</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="L22" s="2"/>
       <c r="M22" t="s" s="2">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3190,7 +3219,7 @@
         <v>75</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -3210,17 +3239,17 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E23" t="s" s="2">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F23" t="s" s="2">
         <v>81</v>
@@ -3238,11 +3267,11 @@
         <v>75</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" t="s" s="2">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3269,11 +3298,13 @@
         <v>75</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z23" t="s" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>75</v>
@@ -3291,7 +3322,7 @@
         <v>75</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
@@ -3309,12 +3340,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24" hidden="true">
+    <row r="24">
       <c r="A24" t="s" s="2">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3322,13 +3353,13 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H24" t="s" s="2">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="I24" t="s" s="2">
         <v>75</v>
@@ -3337,12 +3368,10 @@
         <v>75</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>158</v>
+        <v>86</v>
       </c>
       <c r="L24" s="2"/>
-      <c r="M24" t="s" s="2">
-        <v>159</v>
-      </c>
+      <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
@@ -3368,13 +3397,11 @@
         <v>75</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y24" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>75</v>
+        <v>152</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>75</v>
@@ -3392,10 +3419,10 @@
         <v>75</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>76</v>
@@ -3412,10 +3439,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3441,17 +3468,15 @@
         <v>86</v>
       </c>
       <c r="L25" s="2"/>
-      <c r="M25" t="s" s="2">
-        <v>162</v>
-      </c>
+      <c r="M25" s="2"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
-        <v>163</v>
+        <v>75</v>
       </c>
       <c r="Q25" s="2"/>
       <c r="R25" t="s" s="2">
-        <v>75</v>
+        <v>154</v>
       </c>
       <c r="S25" t="s" s="2">
         <v>75</v>
@@ -3473,7 +3498,7 @@
       </c>
       <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>75</v>
@@ -3491,7 +3516,7 @@
         <v>75</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
@@ -3509,20 +3534,18 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E26" t="s" s="2">
-        <v>167</v>
-      </c>
+      <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
         <v>81</v>
       </c>
@@ -3530,7 +3553,7 @@
         <v>76</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>146</v>
+        <v>75</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>75</v>
@@ -3539,12 +3562,10 @@
         <v>75</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="L26" s="2"/>
-      <c r="M26" t="s" s="2">
-        <v>169</v>
-      </c>
+      <c r="M26" s="2"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -3594,7 +3615,7 @@
         <v>75</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>81</v>
@@ -3612,20 +3633,18 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" hidden="true">
+    <row r="27">
       <c r="A27" t="s" s="2">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E27" t="s" s="2">
-        <v>172</v>
-      </c>
+      <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
         <v>81</v>
       </c>
@@ -3633,7 +3652,7 @@
         <v>76</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>75</v>
@@ -3642,11 +3661,13 @@
         <v>75</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="L27" s="2"/>
+        <v>159</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>160</v>
+      </c>
       <c r="M27" t="s" s="2">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3697,7 +3718,7 @@
         <v>75</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
@@ -3717,17 +3738,17 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E28" t="s" s="2">
-        <v>177</v>
+        <v>85</v>
       </c>
       <c r="F28" t="s" s="2">
         <v>81</v>
@@ -3745,11 +3766,11 @@
         <v>75</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>178</v>
+        <v>86</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" t="s" s="2">
-        <v>179</v>
+        <v>87</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3776,13 +3797,11 @@
         <v>75</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y28" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y28" s="2"/>
       <c r="Z28" t="s" s="2">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>75</v>
@@ -3800,7 +3819,7 @@
         <v>75</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
@@ -3818,20 +3837,18 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E29" t="s" s="2">
-        <v>182</v>
-      </c>
+      <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
         <v>81</v>
       </c>
@@ -3839,7 +3856,7 @@
         <v>76</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>146</v>
+        <v>75</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>75</v>
@@ -3848,11 +3865,11 @@
         <v>75</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" t="s" s="2">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3903,7 +3920,7 @@
         <v>75</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
@@ -3923,10 +3940,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -3949,14 +3966,16 @@
         <v>75</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>152</v>
+        <v>86</v>
       </c>
       <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
+      <c r="M30" t="s" s="2">
+        <v>167</v>
+      </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
-        <v>75</v>
+        <v>168</v>
       </c>
       <c r="Q30" s="2"/>
       <c r="R30" t="s" s="2">
@@ -3978,13 +3997,11 @@
         <v>75</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y30" s="2"/>
       <c r="Z30" t="s" s="2">
-        <v>75</v>
+        <v>169</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>75</v>
@@ -4002,7 +4019,7 @@
         <v>75</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>81</v>
@@ -4022,24 +4039,26 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E31" s="2"/>
+      <c r="E31" t="s" s="2">
+        <v>172</v>
+      </c>
       <c r="F31" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>75</v>
@@ -4048,13 +4067,11 @@
         <v>75</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="L31" t="s" s="2">
-        <v>188</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="L31" s="2"/>
       <c r="M31" t="s" s="2">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4105,26 +4122,537 @@
         <v>75</v>
       </c>
       <c r="AF31" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AG31" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI31" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ31" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK31" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" hidden="true">
+      <c r="A32" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="B32" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E32" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="F32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="H32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K32" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="L32" s="2"/>
+      <c r="M32" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="N32" s="2"/>
+      <c r="O32" s="2"/>
+      <c r="P32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q32" s="2"/>
+      <c r="R32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF32" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="AG32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK32" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" hidden="true">
+      <c r="A33" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E33" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="F33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="H33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K33" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="L33" s="2"/>
+      <c r="M33" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
+      <c r="P33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q33" s="2"/>
+      <c r="R33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF33" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK33" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="AG31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI31" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ31" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK31" t="s" s="2">
+      <c r="B34" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E34" t="s" s="2">
+        <v>187</v>
+      </c>
+      <c r="F34" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="H34" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="I34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K34" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="L34" s="2"/>
+      <c r="M34" t="s" s="2">
+        <v>188</v>
+      </c>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
+      <c r="P34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q34" s="2"/>
+      <c r="R34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF34" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="AG34" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK34" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" hidden="true">
+      <c r="A35" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="B35" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G35" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="H35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K35" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q35" s="2"/>
+      <c r="R35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF35" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="AG35" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH35" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK35" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E36" s="2"/>
+      <c r="F36" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G36" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="H36" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="I36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K36" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="L36" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="M36" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q36" s="2"/>
+      <c r="R36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF36" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="AG36" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH36" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AI36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ36" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK36" t="s" s="2">
         <v>75</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK31">
+  <autoFilter ref="A1:AK36">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -4134,7 +4662,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI30">
+  <conditionalFormatting sqref="A2:AI35">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>